<commit_message>
Nose Dock H5-H6 R3.2: hoja sismica con el ANL R3.2.1 y factores del espectro
- Hoja (sobre el original del usuario, solo valores): 43 modos del ANL
  con masa en punta de columnas y tensores activos en el modal,
  W = 12,887.12 kg, T = 0.6248 s. Participacion: X 92.89 %, Z 95.22 %
  con 43 modos (95.97 / 97.59 % con los 80 del ANL).
- STD: factores del espectro de la hoja, X 1.0960 y Z 1.0237
  (antes 1.0961 y 1.0107). DOMINANT 1 y 3 coinciden con los modos
  dominantes.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01C6kEsteTYPJ6UMnzs1Av1k
</commit_message>
<xml_diff>
--- a/002_SISMO_VIENTO_SALVADOR_3.2.xlsx
+++ b/002_SISMO_VIENTO_SALVADOR_3.2.xlsx
@@ -6685,7 +6685,7 @@
         <v>68</v>
       </c>
       <c r="F137" s="36">
-        <v>0.90019</v>
+        <v>0.6248</v>
       </c>
       <c r="G137" t="s">
         <v>66</v>
@@ -6697,7 +6697,7 @@
       </c>
       <c r="F139" s="52">
         <f>P33*Q85*P55/P99*(P57/MAX(P57,MIN(F137,6*P57)))^(2/3)</f>
-        <v>0.130806075766931</v>
+        <v>0.166861710942371</v>
       </c>
     </row>
     <row r="140" spans="4:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3"/>
@@ -6716,7 +6716,7 @@
       </c>
       <c r="F143" s="54">
         <f>MAX(F141,F139)</f>
-        <v>0.137142857142857</v>
+        <v>0.166861710942371</v>
       </c>
     </row>
     <row r="148" spans="2:25" s="39" customFormat="1" x14ac:dyDescent="0.3"/>
@@ -6840,14 +6840,14 @@
         <v>87</v>
       </c>
       <c r="E165" s="82">
-        <v>12780.46</v>
+        <v>12887.12</v>
       </c>
       <c r="F165" s="1" t="s">
         <v>85</v>
       </c>
       <c r="G165" s="55">
         <f>E165/1000</f>
-        <v>12.78046</v>
+        <v>12.88712</v>
       </c>
       <c r="H165" s="1" t="s">
         <v>86</v>
@@ -6858,14 +6858,14 @@
         <v>88</v>
       </c>
       <c r="E166" s="82">
-        <v>12780.46</v>
+        <v>12887.12</v>
       </c>
       <c r="F166" s="1" t="s">
         <v>85</v>
       </c>
       <c r="G166" s="55">
         <f>E166/1000</f>
-        <v>12.78046</v>
+        <v>12.88712</v>
       </c>
       <c r="H166" s="1" t="s">
         <v>86</v>
@@ -6902,7 +6902,7 @@
       </c>
       <c r="G170" s="51">
         <f>G168*G165</f>
-        <v>2.190936</v>
+        <v>2.20922057142857</v>
       </c>
       <c r="H170" s="1" t="s">
         <v>86</v>
@@ -6919,7 +6919,7 @@
       </c>
       <c r="G171" s="51">
         <f>G168*G166</f>
-        <v>2.190936</v>
+        <v>2.20922057142857</v>
       </c>
       <c r="H171" s="1" t="s">
         <v>86</v>
@@ -7031,13 +7031,13 @@
         <v>1</v>
       </c>
       <c r="C177" s="28">
-        <v>1.111</v>
+        <v>1.601</v>
       </c>
       <c r="D177" s="64">
-        <v>0.90019</v>
+        <v>0.6248</v>
       </c>
       <c r="E177" s="28">
-        <v>60.29</v>
+        <v>81.95</v>
       </c>
       <c r="F177" s="28">
         <v>0.0</v>
@@ -7050,15 +7050,15 @@
       </c>
       <c r="I177" s="29">
         <f>ROUND(D177,2)</f>
-        <v>0.9</v>
+        <v>0.62</v>
       </c>
       <c r="J177" s="31">
         <f>VLOOKUP(I177,$H$252:$I$551,2,0)</f>
-        <v>0.130824484863238</v>
+        <v>0.167721825228907</v>
       </c>
       <c r="K177" s="32">
         <f>J177*$K$222*E177/100</f>
-        <v>1008.04704906699</v>
+        <v>1771.30933079787</v>
       </c>
       <c r="L177" s="34">
         <f>J177*$K$223*G177/100</f>
@@ -7080,38 +7080,38 @@
         <v>2</v>
       </c>
       <c r="C178" s="28">
-        <v>1.468</v>
+        <v>2.362</v>
       </c>
       <c r="D178" s="64">
-        <v>0.68123</v>
+        <v>0.4233</v>
       </c>
       <c r="E178" s="28">
-        <v>5.4</v>
+        <v>4.39</v>
       </c>
       <c r="F178" s="28">
         <v>0.0</v>
       </c>
       <c r="G178" s="28">
-        <v>0.0</v>
+        <v>0.19</v>
       </c>
       <c r="H178" s="28" t="s">
         <v>113</v>
       </c>
       <c r="I178" s="29">
         <f t="shared" ref="I178" si="0">ROUND(D178,2)</f>
-        <v>0.68</v>
+        <v>0.42</v>
       </c>
       <c r="J178" s="31">
         <f>VLOOKUP(I178,$H$252:$I$551,2,0)</f>
-        <v>0.157704746439153</v>
+        <v>0.171428571428571</v>
       </c>
       <c r="K178" s="32">
         <f>J178*$K$222*E178/100</f>
-        <v>108.83911699849</v>
+        <v>96.9847830857143</v>
       </c>
       <c r="L178" s="34">
         <f>J178*$K$223*G178/100</f>
-        <v>0</v>
+        <v>4.19751908571429</v>
       </c>
       <c r="N178" s="10" t="s">
         <v>115</v>
@@ -7129,26 +7129,26 @@
         <v>3</v>
       </c>
       <c r="C179" s="28">
-        <v>1.724</v>
+        <v>2.516</v>
       </c>
       <c r="D179" s="64">
-        <v>0.5802</v>
+        <v>0.39738</v>
       </c>
       <c r="E179" s="28">
-        <v>0.0</v>
+        <v>0.01</v>
       </c>
       <c r="F179" s="28">
         <v>0.0</v>
       </c>
       <c r="G179" s="28">
-        <v>50.47</v>
+        <v>87.87</v>
       </c>
       <c r="H179" s="28" t="s">
         <v>113</v>
       </c>
       <c r="I179" s="29">
         <f t="shared" ref="I179" si="1">ROUND(D179,2)</f>
-        <v>0.58</v>
+        <v>0.4</v>
       </c>
       <c r="J179" s="31">
         <f t="shared" ref="J179" si="2">VLOOKUP(I179,$H$252:$I$551,2,0)</f>
@@ -7156,11 +7156,11 @@
       </c>
       <c r="K179" s="32">
         <f t="shared" ref="K179" si="3">J179*$K$222*E179/100</f>
-        <v>0</v>
+        <v>0.220922057142857</v>
       </c>
       <c r="L179" s="34">
         <f t="shared" ref="L179" si="4">J179*$K$223*G179/100</f>
-        <v>1105.7653992</v>
+        <v>1941.24211611429</v>
       </c>
       <c r="N179" s="10"/>
       <c r="O179" s="26"/>
@@ -7170,26 +7170,26 @@
         <v>4</v>
       </c>
       <c r="C180" s="28">
-        <v>1.95</v>
+        <v>3.439</v>
       </c>
       <c r="D180" s="64">
-        <v>0.51273</v>
+        <v>0.29077</v>
       </c>
       <c r="E180" s="28">
-        <v>7.69</v>
+        <v>0.0</v>
       </c>
       <c r="F180" s="28">
         <v>0.0</v>
       </c>
       <c r="G180" s="28">
-        <v>0.0</v>
+        <v>0.6</v>
       </c>
       <c r="H180" s="28" t="s">
         <v>113</v>
       </c>
       <c r="I180" s="29">
         <f t="shared" ref="I180:I219" si="5">ROUND(D180,2)</f>
-        <v>0.51</v>
+        <v>0.29</v>
       </c>
       <c r="J180" s="31">
         <f t="shared" ref="J180:J219" si="6">VLOOKUP(I180,$H$252:$I$551,2,0)</f>
@@ -7197,11 +7197,11 @@
       </c>
       <c r="K180" s="32">
         <f t="shared" ref="K180:K219" si="7">J180*$K$222*E180/100</f>
-        <v>168.4829784</v>
+        <v>0</v>
       </c>
       <c r="L180" s="34">
         <f t="shared" ref="L180:L219" si="8">J180*$K$223*G180/100</f>
-        <v>0</v>
+        <v>13.2553234285714</v>
       </c>
       <c r="N180" s="10"/>
       <c r="O180" s="26"/>
@@ -7211,26 +7211,26 @@
         <v>5</v>
       </c>
       <c r="C181" s="28">
-        <v>2.367</v>
+        <v>3.597</v>
       </c>
       <c r="D181" s="64">
-        <v>0.42248</v>
+        <v>0.278</v>
       </c>
       <c r="E181" s="28">
-        <v>0.0</v>
+        <v>0.39</v>
       </c>
       <c r="F181" s="28">
         <v>0.0</v>
       </c>
       <c r="G181" s="28">
-        <v>26.93</v>
+        <v>0.18</v>
       </c>
       <c r="H181" s="28" t="s">
         <v>113</v>
       </c>
       <c r="I181" s="29">
         <f t="shared" si="5"/>
-        <v>0.42</v>
+        <v>0.28</v>
       </c>
       <c r="J181" s="31">
         <f t="shared" si="6"/>
@@ -7238,11 +7238,11 @@
       </c>
       <c r="K181" s="32">
         <f t="shared" si="7"/>
-        <v>0</v>
+        <v>8.61596022857143</v>
       </c>
       <c r="L181" s="34">
         <f t="shared" si="8"/>
-        <v>590.0190648</v>
+        <v>3.97659702857143</v>
       </c>
       <c r="N181" s="10"/>
       <c r="O181" s="26"/>
@@ -7252,26 +7252,26 @@
         <v>6</v>
       </c>
       <c r="C182" s="28">
-        <v>2.641</v>
+        <v>3.959</v>
       </c>
       <c r="D182" s="64">
-        <v>0.37867</v>
+        <v>0.25258</v>
       </c>
       <c r="E182" s="28">
-        <v>0.0</v>
+        <v>0.08</v>
       </c>
       <c r="F182" s="28">
         <v>0.0</v>
       </c>
       <c r="G182" s="28">
-        <v>0.31</v>
+        <v>2.49</v>
       </c>
       <c r="H182" s="28" t="s">
         <v>113</v>
       </c>
       <c r="I182" s="29">
         <f t="shared" si="5"/>
-        <v>0.38</v>
+        <v>0.25</v>
       </c>
       <c r="J182" s="31">
         <f t="shared" si="6"/>
@@ -7279,11 +7279,11 @@
       </c>
       <c r="K182" s="32">
         <f t="shared" si="7"/>
-        <v>0</v>
+        <v>1.76737645714286</v>
       </c>
       <c r="L182" s="34">
         <f t="shared" si="8"/>
-        <v>6.7919016</v>
+        <v>55.0095922285715</v>
       </c>
       <c r="N182" s="10"/>
       <c r="O182" s="26"/>
@@ -7293,26 +7293,26 @@
         <v>7</v>
       </c>
       <c r="C183" s="28">
-        <v>2.732</v>
+        <v>4.965</v>
       </c>
       <c r="D183" s="64">
-        <v>0.36606</v>
+        <v>0.20142</v>
       </c>
       <c r="E183" s="28">
-        <v>0.12</v>
+        <v>0.2</v>
       </c>
       <c r="F183" s="28">
         <v>0.0</v>
       </c>
       <c r="G183" s="28">
-        <v>0.0</v>
+        <v>1.12</v>
       </c>
       <c r="H183" s="28" t="s">
         <v>113</v>
       </c>
       <c r="I183" s="29">
         <f t="shared" si="5"/>
-        <v>0.37</v>
+        <v>0.2</v>
       </c>
       <c r="J183" s="31">
         <f t="shared" si="6"/>
@@ -7320,11 +7320,11 @@
       </c>
       <c r="K183" s="32">
         <f t="shared" si="7"/>
-        <v>2.6291232</v>
+        <v>4.41844114285714</v>
       </c>
       <c r="L183" s="34">
         <f t="shared" si="8"/>
-        <v>0</v>
+        <v>24.7432704</v>
       </c>
       <c r="N183" s="10"/>
       <c r="O183" s="26"/>
@@ -7334,38 +7334,38 @@
         <v>8</v>
       </c>
       <c r="C184" s="28">
-        <v>3.604</v>
+        <v>5.135</v>
       </c>
       <c r="D184" s="64">
-        <v>0.27745</v>
+        <v>0.19473</v>
       </c>
       <c r="E184" s="28">
-        <v>0.0</v>
+        <v>0.1</v>
       </c>
       <c r="F184" s="28">
         <v>0.0</v>
       </c>
       <c r="G184" s="28">
-        <v>5.31</v>
+        <v>0.7</v>
       </c>
       <c r="H184" s="28" t="s">
         <v>113</v>
       </c>
       <c r="I184" s="29">
         <f t="shared" si="5"/>
-        <v>0.28</v>
+        <v>0.19</v>
       </c>
       <c r="J184" s="31">
         <f t="shared" si="6"/>
-        <v>0.171428571428571</v>
+        <v>0.165714285714286</v>
       </c>
       <c r="K184" s="32">
         <f t="shared" si="7"/>
-        <v>0</v>
+        <v>2.13557988571429</v>
       </c>
       <c r="L184" s="34">
         <f t="shared" si="8"/>
-        <v>116.3387016</v>
+        <v>14.9490592</v>
       </c>
       <c r="N184" s="10"/>
       <c r="O184" s="26"/>
@@ -7375,38 +7375,38 @@
         <v>9</v>
       </c>
       <c r="C185" s="28">
-        <v>3.824</v>
+        <v>5.913</v>
       </c>
       <c r="D185" s="64">
-        <v>0.2615</v>
+        <v>0.16911</v>
       </c>
       <c r="E185" s="28">
-        <v>4.58</v>
+        <v>0.0</v>
       </c>
       <c r="F185" s="28">
         <v>0.0</v>
       </c>
       <c r="G185" s="28">
-        <v>0.0</v>
+        <v>0.34</v>
       </c>
       <c r="H185" s="28" t="s">
         <v>113</v>
       </c>
       <c r="I185" s="29">
         <f t="shared" si="5"/>
-        <v>0.26</v>
+        <v>0.17</v>
       </c>
       <c r="J185" s="31">
         <f t="shared" si="6"/>
-        <v>0.171428571428571</v>
+        <v>0.154285714285714</v>
       </c>
       <c r="K185" s="32">
         <f t="shared" si="7"/>
-        <v>100.3448688</v>
+        <v>0</v>
       </c>
       <c r="L185" s="34">
         <f t="shared" si="8"/>
-        <v>0</v>
+        <v>6.76021494857143</v>
       </c>
       <c r="N185" s="10"/>
     </row>
@@ -7415,38 +7415,38 @@
         <v>10</v>
       </c>
       <c r="C186" s="28">
-        <v>4.235</v>
+        <v>7.071</v>
       </c>
       <c r="D186" s="64">
-        <v>0.23613</v>
+        <v>0.14143</v>
       </c>
       <c r="E186" s="28">
-        <v>0.04</v>
+        <v>0.0</v>
       </c>
       <c r="F186" s="28">
         <v>0.0</v>
       </c>
       <c r="G186" s="28">
-        <v>0.03</v>
+        <v>0.14</v>
       </c>
       <c r="H186" s="28" t="s">
         <v>113</v>
       </c>
       <c r="I186" s="29">
         <f t="shared" si="5"/>
-        <v>0.24</v>
+        <v>0.14</v>
       </c>
       <c r="J186" s="31">
         <f t="shared" si="6"/>
-        <v>0.171428571428571</v>
+        <v>0.137142857142857</v>
       </c>
       <c r="K186" s="32">
         <f t="shared" si="7"/>
-        <v>0.8763744</v>
+        <v>0</v>
       </c>
       <c r="L186" s="34">
         <f t="shared" si="8"/>
-        <v>0.6572808</v>
+        <v>2.47432704</v>
       </c>
       <c r="N186" s="10"/>
     </row>
@@ -7455,10 +7455,10 @@
         <v>11</v>
       </c>
       <c r="C187" s="28">
-        <v>4.767</v>
+        <v>7.257</v>
       </c>
       <c r="D187" s="64">
-        <v>0.20976</v>
+        <v>0.13779</v>
       </c>
       <c r="E187" s="28">
         <v>0.0</v>
@@ -7467,18 +7467,18 @@
         <v>0.0</v>
       </c>
       <c r="G187" s="28">
-        <v>1.89</v>
+        <v>0.03</v>
       </c>
       <c r="H187" s="28" t="s">
         <v>113</v>
       </c>
       <c r="I187" s="29">
         <f t="shared" si="5"/>
-        <v>0.21</v>
+        <v>0.14</v>
       </c>
       <c r="J187" s="31">
         <f t="shared" si="6"/>
-        <v>0.171428571428571</v>
+        <v>0.137142857142857</v>
       </c>
       <c r="K187" s="32">
         <f t="shared" si="7"/>
@@ -7486,7 +7486,7 @@
       </c>
       <c r="L187" s="34">
         <f t="shared" si="8"/>
-        <v>41.4086904</v>
+        <v>0.530212937142857</v>
       </c>
       <c r="N187" s="59" t="s">
         <v>116</v>
@@ -7497,10 +7497,10 @@
         <v>12</v>
       </c>
       <c r="C188" s="28">
-        <v>5.243</v>
+        <v>7.513</v>
       </c>
       <c r="D188" s="64">
-        <v>0.19073</v>
+        <v>0.13311</v>
       </c>
       <c r="E188" s="28">
         <v>0.0</v>
@@ -7509,18 +7509,18 @@
         <v>0.0</v>
       </c>
       <c r="G188" s="28">
-        <v>1.46</v>
+        <v>0.05</v>
       </c>
       <c r="H188" s="28" t="s">
         <v>113</v>
       </c>
       <c r="I188" s="29">
         <f t="shared" si="5"/>
-        <v>0.19</v>
+        <v>0.13</v>
       </c>
       <c r="J188" s="31">
         <f t="shared" si="6"/>
-        <v>0.165714285714286</v>
+        <v>0.131428571428571</v>
       </c>
       <c r="K188" s="32">
         <f t="shared" si="7"/>
@@ -7528,7 +7528,7 @@
       </c>
       <c r="L188" s="34">
         <f t="shared" si="8"/>
-        <v>30.92141008</v>
+        <v>0.846867885714286</v>
       </c>
       <c r="N188" s="10" t="s">
         <v>114</v>
@@ -7561,38 +7561,38 @@
         <v>13</v>
       </c>
       <c r="C189" s="28">
-        <v>5.801</v>
+        <v>7.756</v>
       </c>
       <c r="D189" s="64">
-        <v>0.17239</v>
+        <v>0.12893</v>
       </c>
       <c r="E189" s="28">
-        <v>0.0</v>
+        <v>0.01</v>
       </c>
       <c r="F189" s="28">
         <v>0.0</v>
       </c>
       <c r="G189" s="28">
-        <v>0.78</v>
+        <v>0.09</v>
       </c>
       <c r="H189" s="28" t="s">
         <v>113</v>
       </c>
       <c r="I189" s="29">
         <f t="shared" si="5"/>
-        <v>0.17</v>
+        <v>0.13</v>
       </c>
       <c r="J189" s="31">
         <f t="shared" si="6"/>
-        <v>0.154285714285714</v>
+        <v>0.131428571428571</v>
       </c>
       <c r="K189" s="32">
         <f t="shared" si="7"/>
-        <v>0</v>
+        <v>0.169373577142857</v>
       </c>
       <c r="L189" s="34">
         <f t="shared" si="8"/>
-        <v>15.38037072</v>
+        <v>1.52436219428571</v>
       </c>
       <c r="N189" s="10" t="s">
         <v>115</v>
@@ -7634,38 +7634,38 @@
         <v>14</v>
       </c>
       <c r="C190" s="28">
-        <v>5.999</v>
+        <v>8.651</v>
       </c>
       <c r="D190" s="64">
-        <v>0.16669</v>
+        <v>0.11559</v>
       </c>
       <c r="E190" s="28">
-        <v>0.06</v>
+        <v>0.01</v>
       </c>
       <c r="F190" s="28">
         <v>0.0</v>
       </c>
       <c r="G190" s="28">
-        <v>0.04</v>
+        <v>0.2</v>
       </c>
       <c r="H190" s="28" t="s">
         <v>113</v>
       </c>
       <c r="I190" s="29">
         <f t="shared" si="5"/>
-        <v>0.17</v>
+        <v>0.12</v>
       </c>
       <c r="J190" s="31">
         <f t="shared" si="6"/>
-        <v>0.154285714285714</v>
+        <v>0.125714285714286</v>
       </c>
       <c r="K190" s="32">
         <f t="shared" si="7"/>
-        <v>1.18310544</v>
+        <v>0.162009508571429</v>
       </c>
       <c r="L190" s="34">
         <f t="shared" si="8"/>
-        <v>0.78873696</v>
+        <v>3.24019017142857</v>
       </c>
       <c r="N190" s="10"/>
       <c r="T190">
@@ -7698,13 +7698,13 @@
         <v>15</v>
       </c>
       <c r="C191" s="28">
-        <v>6.299</v>
+        <v>9.279</v>
       </c>
       <c r="D191" s="64">
-        <v>0.15876</v>
+        <v>0.10777</v>
       </c>
       <c r="E191" s="28">
-        <v>3.72</v>
+        <v>0.04</v>
       </c>
       <c r="F191" s="28">
         <v>0.0</v>
@@ -7717,15 +7717,15 @@
       </c>
       <c r="I191" s="29">
         <f t="shared" si="5"/>
-        <v>0.16</v>
+        <v>0.11</v>
       </c>
       <c r="J191" s="31">
         <f t="shared" si="6"/>
-        <v>0.148571428571429</v>
+        <v>0.12</v>
       </c>
       <c r="K191" s="32">
         <f t="shared" si="7"/>
-        <v>70.63577664</v>
+        <v>0.61858176</v>
       </c>
       <c r="L191" s="34">
         <f t="shared" si="8"/>
@@ -7762,10 +7762,10 @@
         <v>16</v>
       </c>
       <c r="C192" s="28">
-        <v>6.766</v>
+        <v>9.561</v>
       </c>
       <c r="D192" s="64">
-        <v>0.14781</v>
+        <v>0.1046</v>
       </c>
       <c r="E192" s="28">
         <v>0.0</v>
@@ -7774,18 +7774,18 @@
         <v>0.0</v>
       </c>
       <c r="G192" s="28">
-        <v>0.0</v>
+        <v>0.49</v>
       </c>
       <c r="H192" s="28" t="s">
         <v>113</v>
       </c>
       <c r="I192" s="29">
         <f t="shared" si="5"/>
-        <v>0.15</v>
+        <v>0.1</v>
       </c>
       <c r="J192" s="31">
         <f t="shared" si="6"/>
-        <v>0.142857142857143</v>
+        <v>0.114285714285714</v>
       </c>
       <c r="K192" s="32">
         <f t="shared" si="7"/>
@@ -7793,7 +7793,7 @@
       </c>
       <c r="L192" s="34">
         <f t="shared" si="8"/>
-        <v>0</v>
+        <v>7.2167872</v>
       </c>
       <c r="N192" s="10"/>
       <c r="T192">
@@ -7826,13 +7826,13 @@
         <v>17</v>
       </c>
       <c r="C193" s="28">
-        <v>6.813</v>
+        <v>9.683</v>
       </c>
       <c r="D193" s="64">
-        <v>0.14678</v>
+        <v>0.10327</v>
       </c>
       <c r="E193" s="28">
-        <v>0.43</v>
+        <v>3.84</v>
       </c>
       <c r="F193" s="28">
         <v>0.0</v>
@@ -7845,15 +7845,15 @@
       </c>
       <c r="I193" s="29">
         <f t="shared" si="5"/>
-        <v>0.15</v>
+        <v>0.1</v>
       </c>
       <c r="J193" s="31">
         <f t="shared" si="6"/>
-        <v>0.142857142857143</v>
+        <v>0.114285714285714</v>
       </c>
       <c r="K193" s="32">
         <f t="shared" si="7"/>
-        <v>7.850854</v>
+        <v>56.5560466285714</v>
       </c>
       <c r="L193" s="34">
         <f t="shared" si="8"/>
@@ -7889,38 +7889,38 @@
         <v>18</v>
       </c>
       <c r="C194" s="28">
-        <v>6.971</v>
+        <v>9.975</v>
       </c>
       <c r="D194" s="64">
-        <v>0.14344</v>
+        <v>0.10025</v>
       </c>
       <c r="E194" s="28">
-        <v>0.16</v>
+        <v>0.01</v>
       </c>
       <c r="F194" s="28">
         <v>0.0</v>
       </c>
       <c r="G194" s="28">
-        <v>0.08</v>
+        <v>0.72</v>
       </c>
       <c r="H194" s="28" t="s">
         <v>113</v>
       </c>
       <c r="I194" s="29">
         <f t="shared" si="5"/>
-        <v>0.14</v>
+        <v>0.1</v>
       </c>
       <c r="J194" s="31">
         <f t="shared" si="6"/>
-        <v>0.137142857142857</v>
+        <v>0.114285714285714</v>
       </c>
       <c r="K194" s="32">
         <f t="shared" si="7"/>
-        <v>2.80439808</v>
+        <v>0.147281371428571</v>
       </c>
       <c r="L194" s="34">
         <f t="shared" si="8"/>
-        <v>1.40219904</v>
+        <v>10.6042587428571</v>
       </c>
       <c r="T194">
         <v>5</v>
@@ -7952,38 +7952,38 @@
         <v>19</v>
       </c>
       <c r="C195" s="28">
-        <v>7.268</v>
+        <v>10.192</v>
       </c>
       <c r="D195" s="64">
-        <v>0.13759</v>
+        <v>0.09811</v>
       </c>
       <c r="E195" s="28">
-        <v>4.41</v>
+        <v>0.01</v>
       </c>
       <c r="F195" s="28">
         <v>0.0</v>
       </c>
       <c r="G195" s="28">
-        <v>0.0</v>
+        <v>0.01</v>
       </c>
       <c r="H195" s="28" t="s">
         <v>113</v>
       </c>
       <c r="I195" s="29">
         <f t="shared" si="5"/>
-        <v>0.14</v>
+        <v>0.1</v>
       </c>
       <c r="J195" s="31">
         <f t="shared" si="6"/>
-        <v>0.137142857142857</v>
+        <v>0.114285714285714</v>
       </c>
       <c r="K195" s="32">
         <f t="shared" si="7"/>
-        <v>77.29622208</v>
+        <v>0.147281371428571</v>
       </c>
       <c r="L195" s="34">
         <f t="shared" si="8"/>
-        <v>0</v>
+        <v>0.147281371428571</v>
       </c>
       <c r="T195">
         <v>6</v>
@@ -8015,38 +8015,38 @@
         <v>20</v>
       </c>
       <c r="C196" s="28">
-        <v>7.67</v>
+        <v>10.482</v>
       </c>
       <c r="D196" s="64">
-        <v>0.13038</v>
+        <v>0.0954</v>
       </c>
       <c r="E196" s="28">
-        <v>0.16</v>
+        <v>0.0</v>
       </c>
       <c r="F196" s="28">
         <v>0.0</v>
       </c>
       <c r="G196" s="28">
-        <v>0.01</v>
+        <v>0.0</v>
       </c>
       <c r="H196" s="28" t="s">
         <v>113</v>
       </c>
       <c r="I196" s="29">
         <f t="shared" si="5"/>
-        <v>0.13</v>
+        <v>0.1</v>
       </c>
       <c r="J196" s="31">
         <f t="shared" si="6"/>
-        <v>0.131428571428571</v>
+        <v>0.114285714285714</v>
       </c>
       <c r="K196" s="32">
         <f t="shared" si="7"/>
-        <v>2.68754816</v>
+        <v>0</v>
       </c>
       <c r="L196" s="34">
         <f t="shared" si="8"/>
-        <v>0.16797176</v>
+        <v>0</v>
       </c>
       <c r="T196">
         <v>7</v>
@@ -8078,10 +8078,10 @@
         <v>21</v>
       </c>
       <c r="C197" s="28">
-        <v>7.716</v>
+        <v>10.748</v>
       </c>
       <c r="D197" s="64">
-        <v>0.1296</v>
+        <v>0.09304</v>
       </c>
       <c r="E197" s="28">
         <v>0.02</v>
@@ -8097,15 +8097,15 @@
       </c>
       <c r="I197" s="29">
         <f t="shared" si="5"/>
-        <v>0.13</v>
+        <v>0.09</v>
       </c>
       <c r="J197" s="31">
         <f t="shared" si="6"/>
-        <v>0.131428571428571</v>
+        <v>0.108571428571429</v>
       </c>
       <c r="K197" s="32">
         <f t="shared" si="7"/>
-        <v>0.33594352</v>
+        <v>0.279834605714286</v>
       </c>
       <c r="L197" s="34">
         <f t="shared" si="8"/>
@@ -8141,13 +8141,13 @@
         <v>22</v>
       </c>
       <c r="C198" s="28">
-        <v>7.74</v>
+        <v>10.829</v>
       </c>
       <c r="D198" s="64">
-        <v>0.1292</v>
+        <v>0.09234</v>
       </c>
       <c r="E198" s="28">
-        <v>0.06</v>
+        <v>0.04</v>
       </c>
       <c r="F198" s="28">
         <v>0.0</v>
@@ -8160,15 +8160,15 @@
       </c>
       <c r="I198" s="29">
         <f t="shared" si="5"/>
-        <v>0.13</v>
+        <v>0.09</v>
       </c>
       <c r="J198" s="31">
         <f t="shared" si="6"/>
-        <v>0.131428571428571</v>
+        <v>0.108571428571429</v>
       </c>
       <c r="K198" s="32">
         <f t="shared" si="7"/>
-        <v>1.00783056</v>
+        <v>0.559669211428572</v>
       </c>
       <c r="L198" s="34">
         <f t="shared" si="8"/>
@@ -8204,13 +8204,13 @@
         <v>23</v>
       </c>
       <c r="C199" s="28">
-        <v>7.784</v>
+        <v>10.884</v>
       </c>
       <c r="D199" s="64">
-        <v>0.12847</v>
+        <v>0.09188</v>
       </c>
       <c r="E199" s="28">
-        <v>0.57</v>
+        <v>0.16</v>
       </c>
       <c r="F199" s="28">
         <v>0.0</v>
@@ -8223,15 +8223,15 @@
       </c>
       <c r="I199" s="29">
         <f t="shared" si="5"/>
-        <v>0.13</v>
+        <v>0.09</v>
       </c>
       <c r="J199" s="31">
         <f t="shared" si="6"/>
-        <v>0.131428571428571</v>
+        <v>0.108571428571429</v>
       </c>
       <c r="K199" s="32">
         <f t="shared" si="7"/>
-        <v>9.57439032</v>
+        <v>2.23867684571429</v>
       </c>
       <c r="L199" s="34">
         <f t="shared" si="8"/>
@@ -8267,13 +8267,13 @@
         <v>24</v>
       </c>
       <c r="C200" s="28">
-        <v>7.794</v>
+        <v>10.933</v>
       </c>
       <c r="D200" s="64">
-        <v>0.1283</v>
+        <v>0.09146</v>
       </c>
       <c r="E200" s="28">
-        <v>0.0</v>
+        <v>0.44</v>
       </c>
       <c r="F200" s="28">
         <v>0.0</v>
@@ -8286,15 +8286,15 @@
       </c>
       <c r="I200" s="29">
         <f t="shared" si="5"/>
-        <v>0.13</v>
+        <v>0.09</v>
       </c>
       <c r="J200" s="31">
         <f t="shared" si="6"/>
-        <v>0.131428571428571</v>
+        <v>0.108571428571429</v>
       </c>
       <c r="K200" s="32">
         <f t="shared" si="7"/>
-        <v>0</v>
+        <v>6.15636132571429</v>
       </c>
       <c r="L200" s="34">
         <f t="shared" si="8"/>
@@ -8330,13 +8330,13 @@
         <v>25</v>
       </c>
       <c r="C201" s="28">
-        <v>7.804</v>
+        <v>10.983</v>
       </c>
       <c r="D201" s="64">
-        <v>0.12814</v>
+        <v>0.09105</v>
       </c>
       <c r="E201" s="28">
-        <v>0.13</v>
+        <v>0.0</v>
       </c>
       <c r="F201" s="28">
         <v>0.0</v>
@@ -8349,15 +8349,15 @@
       </c>
       <c r="I201" s="29">
         <f t="shared" si="5"/>
-        <v>0.13</v>
+        <v>0.09</v>
       </c>
       <c r="J201" s="31">
         <f t="shared" si="6"/>
-        <v>0.131428571428571</v>
+        <v>0.108571428571429</v>
       </c>
       <c r="K201" s="32">
         <f t="shared" si="7"/>
-        <v>2.18363288</v>
+        <v>0</v>
       </c>
       <c r="L201" s="34">
         <f t="shared" si="8"/>
@@ -8393,13 +8393,13 @@
         <v>26</v>
       </c>
       <c r="C202" s="28">
-        <v>7.805</v>
+        <v>10.991</v>
       </c>
       <c r="D202" s="64">
-        <v>0.12811</v>
+        <v>0.09098</v>
       </c>
       <c r="E202" s="28">
-        <v>0.0</v>
+        <v>0.11</v>
       </c>
       <c r="F202" s="28">
         <v>0.0</v>
@@ -8412,15 +8412,15 @@
       </c>
       <c r="I202" s="29">
         <f t="shared" si="5"/>
-        <v>0.13</v>
+        <v>0.09</v>
       </c>
       <c r="J202" s="31">
         <f t="shared" si="6"/>
-        <v>0.131428571428571</v>
+        <v>0.108571428571429</v>
       </c>
       <c r="K202" s="32">
         <f t="shared" si="7"/>
-        <v>0</v>
+        <v>1.53909033142857</v>
       </c>
       <c r="L202" s="34">
         <f t="shared" si="8"/>
@@ -8456,13 +8456,13 @@
         <v>27</v>
       </c>
       <c r="C203" s="28">
-        <v>7.808</v>
+        <v>11.0</v>
       </c>
       <c r="D203" s="64">
-        <v>0.12807</v>
+        <v>0.09091</v>
       </c>
       <c r="E203" s="28">
-        <v>0.04</v>
+        <v>0.0</v>
       </c>
       <c r="F203" s="28">
         <v>0.0</v>
@@ -8475,15 +8475,15 @@
       </c>
       <c r="I203" s="29">
         <f t="shared" si="5"/>
-        <v>0.13</v>
+        <v>0.09</v>
       </c>
       <c r="J203" s="31">
         <f t="shared" si="6"/>
-        <v>0.131428571428571</v>
+        <v>0.108571428571429</v>
       </c>
       <c r="K203" s="32">
         <f t="shared" si="7"/>
-        <v>0.67188704</v>
+        <v>0</v>
       </c>
       <c r="L203" s="34">
         <f t="shared" si="8"/>
@@ -8519,13 +8519,13 @@
         <v>28</v>
       </c>
       <c r="C204" s="28">
-        <v>7.809</v>
+        <v>11.003</v>
       </c>
       <c r="D204" s="64">
-        <v>0.12806</v>
+        <v>0.09088</v>
       </c>
       <c r="E204" s="28">
-        <v>0.0</v>
+        <v>0.05</v>
       </c>
       <c r="F204" s="28">
         <v>0.0</v>
@@ -8538,15 +8538,15 @@
       </c>
       <c r="I204" s="29">
         <f t="shared" si="5"/>
-        <v>0.13</v>
+        <v>0.09</v>
       </c>
       <c r="J204" s="31">
         <f t="shared" si="6"/>
-        <v>0.131428571428571</v>
+        <v>0.108571428571429</v>
       </c>
       <c r="K204" s="32">
         <f t="shared" si="7"/>
-        <v>0</v>
+        <v>0.699586514285714</v>
       </c>
       <c r="L204" s="34">
         <f t="shared" si="8"/>
@@ -8583,13 +8583,13 @@
         <v>29</v>
       </c>
       <c r="C205" s="28">
-        <v>7.81</v>
+        <v>11.005</v>
       </c>
       <c r="D205" s="64">
-        <v>0.12805</v>
+        <v>0.09087</v>
       </c>
       <c r="E205" s="28">
-        <v>0.01</v>
+        <v>0.0</v>
       </c>
       <c r="F205" s="28">
         <v>0.0</v>
@@ -8602,15 +8602,15 @@
       </c>
       <c r="I205" s="29">
         <f t="shared" si="5"/>
-        <v>0.13</v>
+        <v>0.09</v>
       </c>
       <c r="J205" s="31">
         <f t="shared" si="6"/>
-        <v>0.131428571428571</v>
+        <v>0.108571428571429</v>
       </c>
       <c r="K205" s="32">
         <f t="shared" si="7"/>
-        <v>0.16797176</v>
+        <v>0</v>
       </c>
       <c r="L205" s="34">
         <f t="shared" si="8"/>
@@ -8646,10 +8646,10 @@
         <v>30</v>
       </c>
       <c r="C206" s="28">
-        <v>7.81</v>
+        <v>11.006</v>
       </c>
       <c r="D206" s="64">
-        <v>0.12804</v>
+        <v>0.09086</v>
       </c>
       <c r="E206" s="28">
         <v>0.0</v>
@@ -8665,11 +8665,11 @@
       </c>
       <c r="I206" s="29">
         <f t="shared" si="5"/>
-        <v>0.13</v>
+        <v>0.09</v>
       </c>
       <c r="J206" s="31">
         <f t="shared" si="6"/>
-        <v>0.131428571428571</v>
+        <v>0.108571428571429</v>
       </c>
       <c r="K206" s="32">
         <f t="shared" si="7"/>
@@ -8709,13 +8709,13 @@
         <v>31</v>
       </c>
       <c r="C207" s="28">
-        <v>7.914</v>
+        <v>11.006</v>
       </c>
       <c r="D207" s="64">
-        <v>0.12636</v>
+        <v>0.09086</v>
       </c>
       <c r="E207" s="28">
-        <v>0.17</v>
+        <v>0.0</v>
       </c>
       <c r="F207" s="28">
         <v>0.0</v>
@@ -8728,15 +8728,15 @@
       </c>
       <c r="I207" s="29">
         <f t="shared" si="5"/>
-        <v>0.13</v>
+        <v>0.09</v>
       </c>
       <c r="J207" s="31">
         <f t="shared" si="6"/>
-        <v>0.131428571428571</v>
+        <v>0.108571428571429</v>
       </c>
       <c r="K207" s="32">
         <f t="shared" si="7"/>
-        <v>2.85551992</v>
+        <v>0</v>
       </c>
       <c r="L207" s="34">
         <f t="shared" si="8"/>
@@ -8772,13 +8772,13 @@
         <v>32</v>
       </c>
       <c r="C208" s="28">
-        <v>7.945</v>
+        <v>11.008</v>
       </c>
       <c r="D208" s="64">
-        <v>0.12587</v>
+        <v>0.09084</v>
       </c>
       <c r="E208" s="28">
-        <v>0.15</v>
+        <v>0.0</v>
       </c>
       <c r="F208" s="28">
         <v>0.0</v>
@@ -8791,15 +8791,15 @@
       </c>
       <c r="I208" s="29">
         <f t="shared" si="5"/>
-        <v>0.13</v>
+        <v>0.09</v>
       </c>
       <c r="J208" s="31">
         <f t="shared" si="6"/>
-        <v>0.131428571428571</v>
+        <v>0.108571428571429</v>
       </c>
       <c r="K208" s="32">
         <f t="shared" si="7"/>
-        <v>2.5195764</v>
+        <v>0</v>
       </c>
       <c r="L208" s="34">
         <f t="shared" si="8"/>
@@ -8835,13 +8835,13 @@
         <v>33</v>
       </c>
       <c r="C209" s="28">
-        <v>7.96</v>
+        <v>11.059</v>
       </c>
       <c r="D209" s="64">
-        <v>0.12563</v>
+        <v>0.09043</v>
       </c>
       <c r="E209" s="28">
-        <v>0.05</v>
+        <v>0.07</v>
       </c>
       <c r="F209" s="28">
         <v>0.0</v>
@@ -8854,15 +8854,15 @@
       </c>
       <c r="I209" s="29">
         <f t="shared" si="5"/>
-        <v>0.13</v>
+        <v>0.09</v>
       </c>
       <c r="J209" s="31">
         <f t="shared" si="6"/>
-        <v>0.131428571428571</v>
+        <v>0.108571428571429</v>
       </c>
       <c r="K209" s="32">
         <f t="shared" si="7"/>
-        <v>0.8398588</v>
+        <v>0.97942112</v>
       </c>
       <c r="L209" s="34">
         <f t="shared" si="8"/>
@@ -8898,10 +8898,10 @@
         <v>34</v>
       </c>
       <c r="C210" s="28">
-        <v>7.966</v>
+        <v>11.091</v>
       </c>
       <c r="D210" s="64">
-        <v>0.12554</v>
+        <v>0.09016</v>
       </c>
       <c r="E210" s="28">
         <v>0.04</v>
@@ -8917,15 +8917,15 @@
       </c>
       <c r="I210" s="29">
         <f t="shared" si="5"/>
-        <v>0.13</v>
+        <v>0.09</v>
       </c>
       <c r="J210" s="31">
         <f t="shared" si="6"/>
-        <v>0.131428571428571</v>
+        <v>0.108571428571429</v>
       </c>
       <c r="K210" s="32">
         <f t="shared" si="7"/>
-        <v>0.67188704</v>
+        <v>0.559669211428572</v>
       </c>
       <c r="L210" s="34">
         <f t="shared" si="8"/>
@@ -8961,13 +8961,13 @@
         <v>35</v>
       </c>
       <c r="C211" s="28">
-        <v>7.968</v>
+        <v>11.114</v>
       </c>
       <c r="D211" s="64">
-        <v>0.12549</v>
+        <v>0.08998</v>
       </c>
       <c r="E211" s="28">
-        <v>0.01</v>
+        <v>0.07</v>
       </c>
       <c r="F211" s="28">
         <v>0.0</v>
@@ -8980,15 +8980,15 @@
       </c>
       <c r="I211" s="29">
         <f t="shared" si="5"/>
-        <v>0.13</v>
+        <v>0.09</v>
       </c>
       <c r="J211" s="31">
         <f t="shared" si="6"/>
-        <v>0.131428571428571</v>
+        <v>0.108571428571429</v>
       </c>
       <c r="K211" s="32">
         <f t="shared" si="7"/>
-        <v>0.16797176</v>
+        <v>0.97942112</v>
       </c>
       <c r="L211" s="34">
         <f t="shared" si="8"/>
@@ -9024,13 +9024,13 @@
         <v>36</v>
       </c>
       <c r="C212" s="28">
-        <v>7.969</v>
+        <v>11.127</v>
       </c>
       <c r="D212" s="64">
-        <v>0.12548</v>
+        <v>0.08988</v>
       </c>
       <c r="E212" s="28">
-        <v>0.0</v>
+        <v>0.03</v>
       </c>
       <c r="F212" s="28">
         <v>0.0</v>
@@ -9043,15 +9043,15 @@
       </c>
       <c r="I212" s="29">
         <f t="shared" si="5"/>
-        <v>0.13</v>
+        <v>0.09</v>
       </c>
       <c r="J212" s="31">
         <f t="shared" si="6"/>
-        <v>0.131428571428571</v>
+        <v>0.108571428571429</v>
       </c>
       <c r="K212" s="32">
         <f t="shared" si="7"/>
-        <v>0</v>
+        <v>0.419751908571429</v>
       </c>
       <c r="L212" s="34">
         <f t="shared" si="8"/>
@@ -9087,13 +9087,13 @@
         <v>37</v>
       </c>
       <c r="C213" s="28">
-        <v>7.97</v>
+        <v>11.128</v>
       </c>
       <c r="D213" s="64">
-        <v>0.12547</v>
+        <v>0.08987</v>
       </c>
       <c r="E213" s="28">
-        <v>0.0</v>
+        <v>0.05</v>
       </c>
       <c r="F213" s="28">
         <v>0.0</v>
@@ -9106,15 +9106,15 @@
       </c>
       <c r="I213" s="29">
         <f t="shared" si="5"/>
-        <v>0.13</v>
+        <v>0.09</v>
       </c>
       <c r="J213" s="31">
         <f t="shared" si="6"/>
-        <v>0.131428571428571</v>
+        <v>0.108571428571429</v>
       </c>
       <c r="K213" s="32">
         <f t="shared" si="7"/>
-        <v>0</v>
+        <v>0.699586514285714</v>
       </c>
       <c r="L213" s="34">
         <f t="shared" si="8"/>
@@ -9150,13 +9150,13 @@
         <v>38</v>
       </c>
       <c r="C214" s="28">
-        <v>7.986</v>
+        <v>11.13</v>
       </c>
       <c r="D214" s="64">
-        <v>0.12522</v>
+        <v>0.08985</v>
       </c>
       <c r="E214" s="28">
-        <v>0.0</v>
+        <v>0.29</v>
       </c>
       <c r="F214" s="28">
         <v>0.0</v>
@@ -9169,15 +9169,15 @@
       </c>
       <c r="I214" s="29">
         <f t="shared" si="5"/>
-        <v>0.13</v>
+        <v>0.09</v>
       </c>
       <c r="J214" s="31">
         <f t="shared" si="6"/>
-        <v>0.131428571428571</v>
+        <v>0.108571428571429</v>
       </c>
       <c r="K214" s="32">
         <f t="shared" si="7"/>
-        <v>0</v>
+        <v>4.05760178285714</v>
       </c>
       <c r="L214" s="34">
         <f t="shared" si="8"/>
@@ -9213,38 +9213,38 @@
         <v>39</v>
       </c>
       <c r="C215" s="28">
-        <v>8.034</v>
+        <v>11.13</v>
       </c>
       <c r="D215" s="64">
-        <v>0.12447</v>
+        <v>0.08985</v>
       </c>
       <c r="E215" s="28">
-        <v>0.01</v>
+        <v>0.19</v>
       </c>
       <c r="F215" s="28">
         <v>0.0</v>
       </c>
       <c r="G215" s="28">
-        <v>0.09</v>
+        <v>0.0</v>
       </c>
       <c r="H215" s="28" t="s">
         <v>113</v>
       </c>
       <c r="I215" s="29">
         <f t="shared" si="5"/>
-        <v>0.12</v>
+        <v>0.09</v>
       </c>
       <c r="J215" s="31">
         <f t="shared" si="6"/>
-        <v>0.125714285714286</v>
+        <v>0.108571428571429</v>
       </c>
       <c r="K215" s="32">
         <f t="shared" si="7"/>
-        <v>0.16066864</v>
+        <v>2.65842875428571</v>
       </c>
       <c r="L215" s="34">
         <f t="shared" si="8"/>
-        <v>1.44601776</v>
+        <v>0</v>
       </c>
       <c r="T215">
         <v>30</v>
@@ -9276,38 +9276,38 @@
         <v>40</v>
       </c>
       <c r="C216" s="28">
-        <v>8.253</v>
+        <v>11.132</v>
       </c>
       <c r="D216" s="64">
-        <v>0.12117</v>
+        <v>0.08983</v>
       </c>
       <c r="E216" s="28">
-        <v>0.04</v>
+        <v>0.0</v>
       </c>
       <c r="F216" s="28">
         <v>0.0</v>
       </c>
       <c r="G216" s="28">
-        <v>4.28</v>
+        <v>0.0</v>
       </c>
       <c r="H216" s="28" t="s">
         <v>113</v>
       </c>
       <c r="I216" s="29">
         <f t="shared" si="5"/>
-        <v>0.12</v>
+        <v>0.09</v>
       </c>
       <c r="J216" s="31">
         <f t="shared" si="6"/>
-        <v>0.125714285714286</v>
+        <v>0.108571428571429</v>
       </c>
       <c r="K216" s="32">
         <f t="shared" si="7"/>
-        <v>0.64267456</v>
+        <v>0</v>
       </c>
       <c r="L216" s="34">
         <f t="shared" si="8"/>
-        <v>68.76617792</v>
+        <v>0</v>
       </c>
       <c r="T216">
         <v>31</v>
@@ -9339,38 +9339,38 @@
         <v>41</v>
       </c>
       <c r="C217" s="28">
-        <v>8.5</v>
+        <v>11.133</v>
       </c>
       <c r="D217" s="64">
-        <v>0.11764</v>
+        <v>0.08983</v>
       </c>
       <c r="E217" s="28">
-        <v>0.11</v>
+        <v>0.0</v>
       </c>
       <c r="F217" s="28">
         <v>0.0</v>
       </c>
       <c r="G217" s="28">
-        <v>0.74</v>
+        <v>0.0</v>
       </c>
       <c r="H217" s="28" t="s">
         <v>113</v>
       </c>
       <c r="I217" s="29">
         <f t="shared" si="5"/>
-        <v>0.12</v>
+        <v>0.09</v>
       </c>
       <c r="J217" s="31">
         <f t="shared" si="6"/>
-        <v>0.125714285714286</v>
+        <v>0.108571428571429</v>
       </c>
       <c r="K217" s="32">
         <f t="shared" si="7"/>
-        <v>1.76735504</v>
+        <v>0</v>
       </c>
       <c r="L217" s="34">
         <f t="shared" si="8"/>
-        <v>11.88947936</v>
+        <v>0</v>
       </c>
       <c r="T217">
         <v>32</v>
@@ -9402,10 +9402,10 @@
         <v>42</v>
       </c>
       <c r="C218" s="28">
-        <v>8.659</v>
+        <v>11.133</v>
       </c>
       <c r="D218" s="64">
-        <v>0.11548</v>
+        <v>0.08982</v>
       </c>
       <c r="E218" s="28">
         <v>0.0</v>
@@ -9421,11 +9421,11 @@
       </c>
       <c r="I218" s="29">
         <f t="shared" si="5"/>
-        <v>0.12</v>
+        <v>0.09</v>
       </c>
       <c r="J218" s="31">
         <f t="shared" si="6"/>
-        <v>0.125714285714286</v>
+        <v>0.108571428571429</v>
       </c>
       <c r="K218" s="32">
         <f t="shared" si="7"/>
@@ -9465,38 +9465,38 @@
         <v>43</v>
       </c>
       <c r="C219" s="28">
-        <v>8.799</v>
+        <v>11.305</v>
       </c>
       <c r="D219" s="64">
-        <v>0.11365</v>
+        <v>0.08846</v>
       </c>
       <c r="E219" s="28">
-        <v>0.0</v>
+        <v>0.29</v>
       </c>
       <c r="F219" s="28">
         <v>0.0</v>
       </c>
       <c r="G219" s="28">
-        <v>0.03</v>
+        <v>0.0</v>
       </c>
       <c r="H219" s="28" t="s">
         <v>113</v>
       </c>
       <c r="I219" s="29">
         <f t="shared" si="5"/>
-        <v>0.11</v>
+        <v>0.09</v>
       </c>
       <c r="J219" s="31">
         <f t="shared" si="6"/>
-        <v>0.12</v>
+        <v>0.108571428571429</v>
       </c>
       <c r="K219" s="32">
         <f t="shared" si="7"/>
-        <v>0</v>
+        <v>4.05760178285714</v>
       </c>
       <c r="L219" s="34">
         <f t="shared" si="8"/>
-        <v>0.46009656</v>
+        <v>0</v>
       </c>
       <c r="T219">
         <v>51</v>
@@ -9531,7 +9531,7 @@
       <c r="D220" s="115"/>
       <c r="E220" s="116">
         <f>SUM(E177:E219)</f>
-        <v>88.47</v>
+        <v>92.89</v>
       </c>
       <c r="F220" s="116">
         <f t="shared" ref="F220" si="9">SUM(F177:F219)</f>
@@ -9539,7 +9539,7 @@
       </c>
       <c r="G220" s="116">
         <f>SUM(G177:G219)</f>
-        <v>92.45</v>
+        <v>95.22</v>
       </c>
       <c r="H220" s="143" t="s">
         <v>131</v>
@@ -9548,11 +9548,11 @@
       <c r="J220" s="145"/>
       <c r="K220" s="117">
         <f>SQRT(SUMSQ(K177:K219))</f>
-        <v>1038.08845034276</v>
+        <v>1774.91757738548</v>
       </c>
       <c r="L220" s="117">
         <f>SQRT(SUMSQ(L177:L219))</f>
-        <v>1261.82538627984</v>
+        <v>1942.34961995526</v>
       </c>
       <c r="T220">
         <v>52</v>
@@ -9614,7 +9614,7 @@
       </c>
       <c r="K222" s="30">
         <f>E165</f>
-        <v>12780.46</v>
+        <v>12887.12</v>
       </c>
       <c r="L222" t="s">
         <v>134</v>
@@ -9653,7 +9653,7 @@
       </c>
       <c r="K223" s="30">
         <f>E166</f>
-        <v>12780.46</v>
+        <v>12887.12</v>
       </c>
       <c r="L223" t="s">
         <v>134</v>
@@ -9720,11 +9720,11 @@
       </c>
       <c r="K225" s="30">
         <f>K222*VLOOKUP(MAX(E177:E219),E177:J219,6,0)</f>
-        <v>1671.99709581522</v>
+        <v>2161.45128834395</v>
       </c>
       <c r="L225" s="30">
         <f>K222*VLOOKUP(MAX(G177:G219),G177:J219,4,0)</f>
-        <v>2190.936</v>
+        <v>2209.22057142857</v>
       </c>
       <c r="T225">
         <v>57</v>
@@ -9757,11 +9757,11 @@
       </c>
       <c r="K226" s="30">
         <f>0.9*K225</f>
-        <v>1504.7973862337</v>
+        <v>1945.30615950955</v>
       </c>
       <c r="L226" s="30">
         <f>0.9*L225</f>
-        <v>1971.8424</v>
+        <v>1988.29851428571</v>
       </c>
       <c r="T226">
         <v>58</v>
@@ -9826,11 +9826,11 @@
       </c>
       <c r="K228" s="30">
         <f>K222*G168</f>
-        <v>2190.936</v>
+        <v>2209.22057142857</v>
       </c>
       <c r="L228" s="30">
         <f>K222*G168</f>
-        <v>2190.936</v>
+        <v>2209.22057142857</v>
       </c>
       <c r="T228">
         <v>60</v>
@@ -9863,11 +9863,11 @@
       </c>
       <c r="K229" s="30">
         <f>0.8*K228</f>
-        <v>1752.7488</v>
+        <v>1767.37645714286</v>
       </c>
       <c r="L229" s="30">
         <f>0.8*L228</f>
-        <v>1752.7488</v>
+        <v>1767.37645714286</v>
       </c>
       <c r="T229">
         <v>61</v>
@@ -9956,11 +9956,11 @@
       </c>
       <c r="K232" s="44">
         <f>MAX(K229,K226)</f>
-        <v>1752.7488</v>
+        <v>1945.30615950955</v>
       </c>
       <c r="L232" s="44">
         <f>MAX(L229,L226)</f>
-        <v>1971.8424</v>
+        <v>1988.29851428571</v>
       </c>
       <c r="T232">
         <v>64</v>
@@ -10082,11 +10082,11 @@
       </c>
       <c r="K236" s="47">
         <f>K232/1000</f>
-        <v>1.7527488</v>
+        <v>1.94530615950955</v>
       </c>
       <c r="L236" s="47">
         <f>L232/1000</f>
-        <v>1.9718424</v>
+        <v>1.98829851428571</v>
       </c>
       <c r="T236">
         <v>68</v>
@@ -10119,11 +10119,11 @@
       </c>
       <c r="K237" s="47">
         <f>K220/1000</f>
-        <v>1.03808845034276</v>
+        <v>1.77491757738548</v>
       </c>
       <c r="L237" s="47">
         <f>L220/1000</f>
-        <v>1.26182538627984</v>
+        <v>1.94234961995526</v>
       </c>
       <c r="T237">
         <v>69</v>
@@ -10193,11 +10193,11 @@
       </c>
       <c r="K239" s="86">
         <f>MAX(K236/K237,1)</f>
-        <v>1.68843878324748</v>
+        <v>1.09599802508861</v>
       </c>
       <c r="L239" s="86">
         <f>MAX(L236/L237,1)</f>
-        <v>1.56269038603943</v>
+        <v>1.02365634582899</v>
       </c>
       <c r="T239">
         <v>71</v>
@@ -10256,11 +10256,11 @@
       </c>
       <c r="K241" s="86">
         <f>IF(K226/K220&lt;1,"N/A",K226/K220)</f>
-        <v>1.44958494214711</v>
+        <v>1.09599802508861</v>
       </c>
       <c r="L241" s="86">
         <f>IF(L226/L220&lt;1,"N/A",L226/L220)</f>
-        <v>1.56269038603943</v>
+        <v>1.02365634582899</v>
       </c>
       <c r="T241">
         <v>73</v>
@@ -10316,11 +10316,11 @@
     <row r="243" spans="2:27" x14ac:dyDescent="0.3">
       <c r="K243" s="53">
         <f>K225/K220</f>
-        <v>1.61064993571901</v>
+        <v>1.21777558343179</v>
       </c>
       <c r="L243" s="53">
         <f>L225/L220</f>
-        <v>1.73632265115493</v>
+        <v>1.13739593980998</v>
       </c>
       <c r="T243">
         <v>75</v>

</xml_diff>

<commit_message>
Nose Dock H5-H6 R3.2: hoja y factores con el ANL de la viga del eje 3 empotrada
- Hoja (solo valores): 43 modos, W = 12,887.12 kg, T = 0.6231 s.
  X 92.89 % y Z 95.22 % con 43 modos (95.93 / 97.57 % con 80).
- STD: factores del espectro X 1.0967 y Z 1.0012 (antes 1.0960 y
  1.0237). DOMINANT 1 y 3 siguen coincidiendo con los modos dominantes.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01C6kEsteTYPJ6UMnzs1Av1k
</commit_message>
<xml_diff>
--- a/002_SISMO_VIENTO_SALVADOR_3.2.xlsx
+++ b/002_SISMO_VIENTO_SALVADOR_3.2.xlsx
@@ -6685,7 +6685,7 @@
         <v>68</v>
       </c>
       <c r="F137" s="36">
-        <v>0.6248</v>
+        <v>0.6231</v>
       </c>
       <c r="G137" t="s">
         <v>66</v>
@@ -6697,7 +6697,7 @@
       </c>
       <c r="F139" s="52">
         <f>P33*Q85*P55/P99*(P57/MAX(P57,MIN(F137,6*P57)))^(2/3)</f>
-        <v>0.166861710942371</v>
+        <v>0.167165071641971</v>
       </c>
     </row>
     <row r="140" spans="4:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3"/>
@@ -6716,7 +6716,7 @@
       </c>
       <c r="F143" s="54">
         <f>MAX(F141,F139)</f>
-        <v>0.166861710942371</v>
+        <v>0.167165071641971</v>
       </c>
     </row>
     <row r="148" spans="2:25" s="39" customFormat="1" x14ac:dyDescent="0.3"/>
@@ -7031,13 +7031,13 @@
         <v>1</v>
       </c>
       <c r="C177" s="28">
-        <v>1.601</v>
+        <v>1.605</v>
       </c>
       <c r="D177" s="64">
-        <v>0.6248</v>
+        <v>0.6231</v>
       </c>
       <c r="E177" s="28">
-        <v>81.95</v>
+        <v>81.87</v>
       </c>
       <c r="F177" s="28">
         <v>0.0</v>
@@ -7058,7 +7058,7 @@
       </c>
       <c r="K177" s="32">
         <f>J177*$K$222*E177/100</f>
-        <v>1771.30933079787</v>
+        <v>1769.58016976719</v>
       </c>
       <c r="L177" s="34">
         <f>J177*$K$223*G177/100</f>
@@ -7080,19 +7080,19 @@
         <v>2</v>
       </c>
       <c r="C178" s="28">
-        <v>2.362</v>
+        <v>2.372</v>
       </c>
       <c r="D178" s="64">
-        <v>0.4233</v>
+        <v>0.42159</v>
       </c>
       <c r="E178" s="28">
-        <v>4.39</v>
+        <v>4.86</v>
       </c>
       <c r="F178" s="28">
         <v>0.0</v>
       </c>
       <c r="G178" s="28">
-        <v>0.19</v>
+        <v>0.14</v>
       </c>
       <c r="H178" s="28" t="s">
         <v>113</v>
@@ -7107,11 +7107,11 @@
       </c>
       <c r="K178" s="32">
         <f>J178*$K$222*E178/100</f>
-        <v>96.9847830857143</v>
+        <v>107.368119771429</v>
       </c>
       <c r="L178" s="34">
         <f>J178*$K$223*G178/100</f>
-        <v>4.19751908571429</v>
+        <v>3.0929088</v>
       </c>
       <c r="N178" s="10" t="s">
         <v>115</v>
@@ -7129,26 +7129,26 @@
         <v>3</v>
       </c>
       <c r="C179" s="28">
-        <v>2.516</v>
+        <v>2.542</v>
       </c>
       <c r="D179" s="64">
-        <v>0.39738</v>
+        <v>0.39343</v>
       </c>
       <c r="E179" s="28">
-        <v>0.01</v>
+        <v>0.0</v>
       </c>
       <c r="F179" s="28">
         <v>0.0</v>
       </c>
       <c r="G179" s="28">
-        <v>87.87</v>
+        <v>89.87</v>
       </c>
       <c r="H179" s="28" t="s">
         <v>113</v>
       </c>
       <c r="I179" s="29">
         <f t="shared" ref="I179" si="1">ROUND(D179,2)</f>
-        <v>0.4</v>
+        <v>0.39</v>
       </c>
       <c r="J179" s="31">
         <f t="shared" ref="J179" si="2">VLOOKUP(I179,$H$252:$I$551,2,0)</f>
@@ -7156,11 +7156,11 @@
       </c>
       <c r="K179" s="32">
         <f t="shared" ref="K179" si="3">J179*$K$222*E179/100</f>
-        <v>0.220922057142857</v>
+        <v>0</v>
       </c>
       <c r="L179" s="34">
         <f t="shared" ref="L179" si="4">J179*$K$223*G179/100</f>
-        <v>1941.24211611429</v>
+        <v>1985.42652754286</v>
       </c>
       <c r="N179" s="10"/>
       <c r="O179" s="26"/>
@@ -7170,26 +7170,26 @@
         <v>4</v>
       </c>
       <c r="C180" s="28">
-        <v>3.439</v>
+        <v>3.53</v>
       </c>
       <c r="D180" s="64">
-        <v>0.29077</v>
+        <v>0.2833</v>
       </c>
       <c r="E180" s="28">
-        <v>0.0</v>
+        <v>0.02</v>
       </c>
       <c r="F180" s="28">
         <v>0.0</v>
       </c>
       <c r="G180" s="28">
-        <v>0.6</v>
+        <v>0.0</v>
       </c>
       <c r="H180" s="28" t="s">
         <v>113</v>
       </c>
       <c r="I180" s="29">
         <f t="shared" ref="I180:I219" si="5">ROUND(D180,2)</f>
-        <v>0.29</v>
+        <v>0.28</v>
       </c>
       <c r="J180" s="31">
         <f t="shared" ref="J180:J219" si="6">VLOOKUP(I180,$H$252:$I$551,2,0)</f>
@@ -7197,11 +7197,11 @@
       </c>
       <c r="K180" s="32">
         <f t="shared" ref="K180:K219" si="7">J180*$K$222*E180/100</f>
-        <v>0</v>
+        <v>0.441844114285714</v>
       </c>
       <c r="L180" s="34">
         <f t="shared" ref="L180:L219" si="8">J180*$K$223*G180/100</f>
-        <v>13.2553234285714</v>
+        <v>0</v>
       </c>
       <c r="N180" s="10"/>
       <c r="O180" s="26"/>
@@ -7211,26 +7211,26 @@
         <v>5</v>
       </c>
       <c r="C181" s="28">
-        <v>3.597</v>
+        <v>4.147</v>
       </c>
       <c r="D181" s="64">
-        <v>0.278</v>
+        <v>0.24115</v>
       </c>
       <c r="E181" s="28">
-        <v>0.39</v>
+        <v>0.01</v>
       </c>
       <c r="F181" s="28">
         <v>0.0</v>
       </c>
       <c r="G181" s="28">
-        <v>0.18</v>
+        <v>1.02</v>
       </c>
       <c r="H181" s="28" t="s">
         <v>113</v>
       </c>
       <c r="I181" s="29">
         <f t="shared" si="5"/>
-        <v>0.28</v>
+        <v>0.24</v>
       </c>
       <c r="J181" s="31">
         <f t="shared" si="6"/>
@@ -7238,11 +7238,11 @@
       </c>
       <c r="K181" s="32">
         <f t="shared" si="7"/>
-        <v>8.61596022857143</v>
+        <v>0.220922057142857</v>
       </c>
       <c r="L181" s="34">
         <f t="shared" si="8"/>
-        <v>3.97659702857143</v>
+        <v>22.5340498285714</v>
       </c>
       <c r="N181" s="10"/>
       <c r="O181" s="26"/>
@@ -7252,26 +7252,26 @@
         <v>6</v>
       </c>
       <c r="C182" s="28">
-        <v>3.959</v>
+        <v>4.427</v>
       </c>
       <c r="D182" s="64">
-        <v>0.25258</v>
+        <v>0.22586</v>
       </c>
       <c r="E182" s="28">
-        <v>0.08</v>
+        <v>0.02</v>
       </c>
       <c r="F182" s="28">
         <v>0.0</v>
       </c>
       <c r="G182" s="28">
-        <v>2.49</v>
+        <v>0.33</v>
       </c>
       <c r="H182" s="28" t="s">
         <v>113</v>
       </c>
       <c r="I182" s="29">
         <f t="shared" si="5"/>
-        <v>0.25</v>
+        <v>0.23</v>
       </c>
       <c r="J182" s="31">
         <f t="shared" si="6"/>
@@ -7279,11 +7279,11 @@
       </c>
       <c r="K182" s="32">
         <f t="shared" si="7"/>
-        <v>1.76737645714286</v>
+        <v>0.441844114285714</v>
       </c>
       <c r="L182" s="34">
         <f t="shared" si="8"/>
-        <v>55.0095922285715</v>
+        <v>7.29042788571429</v>
       </c>
       <c r="N182" s="10"/>
       <c r="O182" s="26"/>
@@ -7293,19 +7293,19 @@
         <v>7</v>
       </c>
       <c r="C183" s="28">
-        <v>4.965</v>
+        <v>5.077</v>
       </c>
       <c r="D183" s="64">
-        <v>0.20142</v>
+        <v>0.19695</v>
       </c>
       <c r="E183" s="28">
-        <v>0.2</v>
+        <v>0.03</v>
       </c>
       <c r="F183" s="28">
         <v>0.0</v>
       </c>
       <c r="G183" s="28">
-        <v>1.12</v>
+        <v>1.75</v>
       </c>
       <c r="H183" s="28" t="s">
         <v>113</v>
@@ -7320,11 +7320,11 @@
       </c>
       <c r="K183" s="32">
         <f t="shared" si="7"/>
-        <v>4.41844114285714</v>
+        <v>0.662766171428572</v>
       </c>
       <c r="L183" s="34">
         <f t="shared" si="8"/>
-        <v>24.7432704</v>
+        <v>38.66136</v>
       </c>
       <c r="N183" s="10"/>
       <c r="O183" s="26"/>
@@ -7334,19 +7334,19 @@
         <v>8</v>
       </c>
       <c r="C184" s="28">
-        <v>5.135</v>
+        <v>5.392</v>
       </c>
       <c r="D184" s="64">
-        <v>0.19473</v>
+        <v>0.18546</v>
       </c>
       <c r="E184" s="28">
-        <v>0.1</v>
+        <v>0.35</v>
       </c>
       <c r="F184" s="28">
         <v>0.0</v>
       </c>
       <c r="G184" s="28">
-        <v>0.7</v>
+        <v>0.01</v>
       </c>
       <c r="H184" s="28" t="s">
         <v>113</v>
@@ -7361,11 +7361,11 @@
       </c>
       <c r="K184" s="32">
         <f t="shared" si="7"/>
-        <v>2.13557988571429</v>
+        <v>7.4745296</v>
       </c>
       <c r="L184" s="34">
         <f t="shared" si="8"/>
-        <v>14.9490592</v>
+        <v>0.213557988571429</v>
       </c>
       <c r="N184" s="10"/>
       <c r="O184" s="26"/>
@@ -7375,10 +7375,10 @@
         <v>9</v>
       </c>
       <c r="C185" s="28">
-        <v>5.913</v>
+        <v>5.923</v>
       </c>
       <c r="D185" s="64">
-        <v>0.16911</v>
+        <v>0.16884</v>
       </c>
       <c r="E185" s="28">
         <v>0.0</v>
@@ -7387,7 +7387,7 @@
         <v>0.0</v>
       </c>
       <c r="G185" s="28">
-        <v>0.34</v>
+        <v>0.36</v>
       </c>
       <c r="H185" s="28" t="s">
         <v>113</v>
@@ -7406,7 +7406,7 @@
       </c>
       <c r="L185" s="34">
         <f t="shared" si="8"/>
-        <v>6.76021494857143</v>
+        <v>7.15787465142857</v>
       </c>
       <c r="N185" s="10"/>
     </row>
@@ -7418,7 +7418,7 @@
         <v>7.071</v>
       </c>
       <c r="D186" s="64">
-        <v>0.14143</v>
+        <v>0.14142</v>
       </c>
       <c r="E186" s="28">
         <v>0.0</v>
@@ -7455,10 +7455,10 @@
         <v>11</v>
       </c>
       <c r="C187" s="28">
-        <v>7.257</v>
+        <v>7.258</v>
       </c>
       <c r="D187" s="64">
-        <v>0.13779</v>
+        <v>0.13778</v>
       </c>
       <c r="E187" s="28">
         <v>0.0</v>
@@ -7497,10 +7497,10 @@
         <v>12</v>
       </c>
       <c r="C188" s="28">
-        <v>7.513</v>
+        <v>7.514</v>
       </c>
       <c r="D188" s="64">
-        <v>0.13311</v>
+        <v>0.13309</v>
       </c>
       <c r="E188" s="28">
         <v>0.0</v>
@@ -7561,10 +7561,10 @@
         <v>13</v>
       </c>
       <c r="C189" s="28">
-        <v>7.756</v>
+        <v>7.779</v>
       </c>
       <c r="D189" s="64">
-        <v>0.12893</v>
+        <v>0.12855</v>
       </c>
       <c r="E189" s="28">
         <v>0.01</v>
@@ -7634,10 +7634,10 @@
         <v>14</v>
       </c>
       <c r="C190" s="28">
-        <v>8.651</v>
+        <v>8.656</v>
       </c>
       <c r="D190" s="64">
-        <v>0.11559</v>
+        <v>0.11552</v>
       </c>
       <c r="E190" s="28">
         <v>0.01</v>
@@ -7646,7 +7646,7 @@
         <v>0.0</v>
       </c>
       <c r="G190" s="28">
-        <v>0.2</v>
+        <v>0.21</v>
       </c>
       <c r="H190" s="28" t="s">
         <v>113</v>
@@ -7665,7 +7665,7 @@
       </c>
       <c r="L190" s="34">
         <f t="shared" si="8"/>
-        <v>3.24019017142857</v>
+        <v>3.40219968</v>
       </c>
       <c r="N190" s="10"/>
       <c r="T190">
@@ -7704,7 +7704,7 @@
         <v>0.10777</v>
       </c>
       <c r="E191" s="28">
-        <v>0.04</v>
+        <v>0.03</v>
       </c>
       <c r="F191" s="28">
         <v>0.0</v>
@@ -7725,7 +7725,7 @@
       </c>
       <c r="K191" s="32">
         <f t="shared" si="7"/>
-        <v>0.61858176</v>
+        <v>0.46393632</v>
       </c>
       <c r="L191" s="34">
         <f t="shared" si="8"/>
@@ -7762,19 +7762,19 @@
         <v>16</v>
       </c>
       <c r="C192" s="28">
-        <v>9.561</v>
+        <v>9.587</v>
       </c>
       <c r="D192" s="64">
-        <v>0.1046</v>
+        <v>0.10431</v>
       </c>
       <c r="E192" s="28">
-        <v>0.0</v>
+        <v>0.01</v>
       </c>
       <c r="F192" s="28">
         <v>0.0</v>
       </c>
       <c r="G192" s="28">
-        <v>0.49</v>
+        <v>0.51</v>
       </c>
       <c r="H192" s="28" t="s">
         <v>113</v>
@@ -7789,11 +7789,11 @@
       </c>
       <c r="K192" s="32">
         <f t="shared" si="7"/>
-        <v>0</v>
+        <v>0.147281371428571</v>
       </c>
       <c r="L192" s="34">
         <f t="shared" si="8"/>
-        <v>7.2167872</v>
+        <v>7.51134994285714</v>
       </c>
       <c r="N192" s="10"/>
       <c r="T192">
@@ -7826,13 +7826,13 @@
         <v>17</v>
       </c>
       <c r="C193" s="28">
-        <v>9.683</v>
+        <v>9.696</v>
       </c>
       <c r="D193" s="64">
-        <v>0.10327</v>
+        <v>0.10313</v>
       </c>
       <c r="E193" s="28">
-        <v>3.84</v>
+        <v>3.83</v>
       </c>
       <c r="F193" s="28">
         <v>0.0</v>
@@ -7853,7 +7853,7 @@
       </c>
       <c r="K193" s="32">
         <f t="shared" si="7"/>
-        <v>56.5560466285714</v>
+        <v>56.4087652571429</v>
       </c>
       <c r="L193" s="34">
         <f t="shared" si="8"/>
@@ -7889,10 +7889,10 @@
         <v>18</v>
       </c>
       <c r="C194" s="28">
-        <v>9.975</v>
+        <v>9.98</v>
       </c>
       <c r="D194" s="64">
-        <v>0.10025</v>
+        <v>0.1002</v>
       </c>
       <c r="E194" s="28">
         <v>0.01</v>
@@ -7901,7 +7901,7 @@
         <v>0.0</v>
       </c>
       <c r="G194" s="28">
-        <v>0.72</v>
+        <v>0.7</v>
       </c>
       <c r="H194" s="28" t="s">
         <v>113</v>
@@ -7920,7 +7920,7 @@
       </c>
       <c r="L194" s="34">
         <f t="shared" si="8"/>
-        <v>10.6042587428571</v>
+        <v>10.309696</v>
       </c>
       <c r="T194">
         <v>5</v>
@@ -7952,13 +7952,13 @@
         <v>19</v>
       </c>
       <c r="C195" s="28">
-        <v>10.192</v>
+        <v>10.194</v>
       </c>
       <c r="D195" s="64">
-        <v>0.09811</v>
+        <v>0.09809</v>
       </c>
       <c r="E195" s="28">
-        <v>0.01</v>
+        <v>0.0</v>
       </c>
       <c r="F195" s="28">
         <v>0.0</v>
@@ -7979,7 +7979,7 @@
       </c>
       <c r="K195" s="32">
         <f t="shared" si="7"/>
-        <v>0.147281371428571</v>
+        <v>0</v>
       </c>
       <c r="L195" s="34">
         <f t="shared" si="8"/>
@@ -8141,13 +8141,13 @@
         <v>22</v>
       </c>
       <c r="C198" s="28">
-        <v>10.829</v>
+        <v>10.835</v>
       </c>
       <c r="D198" s="64">
-        <v>0.09234</v>
+        <v>0.0923</v>
       </c>
       <c r="E198" s="28">
-        <v>0.04</v>
+        <v>0.03</v>
       </c>
       <c r="F198" s="28">
         <v>0.0</v>
@@ -8168,7 +8168,7 @@
       </c>
       <c r="K198" s="32">
         <f t="shared" si="7"/>
-        <v>0.559669211428572</v>
+        <v>0.419751908571429</v>
       </c>
       <c r="L198" s="34">
         <f t="shared" si="8"/>
@@ -8204,10 +8204,10 @@
         <v>23</v>
       </c>
       <c r="C199" s="28">
-        <v>10.884</v>
+        <v>10.885</v>
       </c>
       <c r="D199" s="64">
-        <v>0.09188</v>
+        <v>0.09187</v>
       </c>
       <c r="E199" s="28">
         <v>0.16</v>
@@ -8267,10 +8267,10 @@
         <v>24</v>
       </c>
       <c r="C200" s="28">
-        <v>10.933</v>
+        <v>10.935</v>
       </c>
       <c r="D200" s="64">
-        <v>0.09146</v>
+        <v>0.09145</v>
       </c>
       <c r="E200" s="28">
         <v>0.44</v>
@@ -8393,7 +8393,7 @@
         <v>26</v>
       </c>
       <c r="C202" s="28">
-        <v>10.991</v>
+        <v>10.992</v>
       </c>
       <c r="D202" s="64">
         <v>0.09098</v>
@@ -8525,7 +8525,7 @@
         <v>0.09088</v>
       </c>
       <c r="E204" s="28">
-        <v>0.05</v>
+        <v>0.04</v>
       </c>
       <c r="F204" s="28">
         <v>0.0</v>
@@ -8546,7 +8546,7 @@
       </c>
       <c r="K204" s="32">
         <f t="shared" si="7"/>
-        <v>0.699586514285714</v>
+        <v>0.559669211428572</v>
       </c>
       <c r="L204" s="34">
         <f t="shared" si="8"/>
@@ -8772,7 +8772,7 @@
         <v>32</v>
       </c>
       <c r="C208" s="28">
-        <v>11.008</v>
+        <v>11.009</v>
       </c>
       <c r="D208" s="64">
         <v>0.09084</v>
@@ -8835,10 +8835,10 @@
         <v>33</v>
       </c>
       <c r="C209" s="28">
-        <v>11.059</v>
+        <v>11.06</v>
       </c>
       <c r="D209" s="64">
-        <v>0.09043</v>
+        <v>0.09042</v>
       </c>
       <c r="E209" s="28">
         <v>0.07</v>
@@ -8898,13 +8898,13 @@
         <v>34</v>
       </c>
       <c r="C210" s="28">
-        <v>11.091</v>
+        <v>11.093</v>
       </c>
       <c r="D210" s="64">
-        <v>0.09016</v>
+        <v>0.09015</v>
       </c>
       <c r="E210" s="28">
-        <v>0.04</v>
+        <v>0.05</v>
       </c>
       <c r="F210" s="28">
         <v>0.0</v>
@@ -8925,7 +8925,7 @@
       </c>
       <c r="K210" s="32">
         <f t="shared" si="7"/>
-        <v>0.559669211428572</v>
+        <v>0.699586514285714</v>
       </c>
       <c r="L210" s="34">
         <f t="shared" si="8"/>
@@ -8961,13 +8961,13 @@
         <v>35</v>
       </c>
       <c r="C211" s="28">
-        <v>11.114</v>
+        <v>11.115</v>
       </c>
       <c r="D211" s="64">
-        <v>0.08998</v>
+        <v>0.08997</v>
       </c>
       <c r="E211" s="28">
-        <v>0.07</v>
+        <v>0.06</v>
       </c>
       <c r="F211" s="28">
         <v>0.0</v>
@@ -8988,7 +8988,7 @@
       </c>
       <c r="K211" s="32">
         <f t="shared" si="7"/>
-        <v>0.97942112</v>
+        <v>0.839503817142857</v>
       </c>
       <c r="L211" s="34">
         <f t="shared" si="8"/>
@@ -9027,10 +9027,10 @@
         <v>11.127</v>
       </c>
       <c r="D212" s="64">
-        <v>0.08988</v>
+        <v>0.08987</v>
       </c>
       <c r="E212" s="28">
-        <v>0.03</v>
+        <v>0.04</v>
       </c>
       <c r="F212" s="28">
         <v>0.0</v>
@@ -9051,7 +9051,7 @@
       </c>
       <c r="K212" s="32">
         <f t="shared" si="7"/>
-        <v>0.419751908571429</v>
+        <v>0.559669211428572</v>
       </c>
       <c r="L212" s="34">
         <f t="shared" si="8"/>
@@ -9090,10 +9090,10 @@
         <v>11.128</v>
       </c>
       <c r="D213" s="64">
-        <v>0.08987</v>
+        <v>0.08986</v>
       </c>
       <c r="E213" s="28">
-        <v>0.05</v>
+        <v>0.04</v>
       </c>
       <c r="F213" s="28">
         <v>0.0</v>
@@ -9114,7 +9114,7 @@
       </c>
       <c r="K213" s="32">
         <f t="shared" si="7"/>
-        <v>0.699586514285714</v>
+        <v>0.559669211428572</v>
       </c>
       <c r="L213" s="34">
         <f t="shared" si="8"/>
@@ -9156,7 +9156,7 @@
         <v>0.08985</v>
       </c>
       <c r="E214" s="28">
-        <v>0.29</v>
+        <v>0.3</v>
       </c>
       <c r="F214" s="28">
         <v>0.0</v>
@@ -9177,7 +9177,7 @@
       </c>
       <c r="K214" s="32">
         <f t="shared" si="7"/>
-        <v>4.05760178285714</v>
+        <v>4.19751908571429</v>
       </c>
       <c r="L214" s="34">
         <f t="shared" si="8"/>
@@ -9219,7 +9219,7 @@
         <v>0.08985</v>
       </c>
       <c r="E215" s="28">
-        <v>0.19</v>
+        <v>0.18</v>
       </c>
       <c r="F215" s="28">
         <v>0.0</v>
@@ -9240,7 +9240,7 @@
       </c>
       <c r="K215" s="32">
         <f t="shared" si="7"/>
-        <v>2.65842875428571</v>
+        <v>2.51851145142857</v>
       </c>
       <c r="L215" s="34">
         <f t="shared" si="8"/>
@@ -9548,11 +9548,11 @@
       <c r="J220" s="145"/>
       <c r="K220" s="117">
         <f>SQRT(SUMSQ(K177:K219))</f>
-        <v>1774.91757738548</v>
+        <v>1773.77280251396</v>
       </c>
       <c r="L220" s="117">
         <f>SQRT(SUMSQ(L177:L219))</f>
-        <v>1942.34961995526</v>
+        <v>1986.0057222423</v>
       </c>
       <c r="T220">
         <v>52</v>
@@ -10119,11 +10119,11 @@
       </c>
       <c r="K237" s="47">
         <f>K220/1000</f>
-        <v>1.77491757738548</v>
+        <v>1.77377280251396</v>
       </c>
       <c r="L237" s="47">
         <f>L220/1000</f>
-        <v>1.94234961995526</v>
+        <v>1.9860057222423</v>
       </c>
       <c r="T237">
         <v>69</v>
@@ -10160,7 +10160,7 @@
       </c>
       <c r="L238" s="68" t="str">
         <f>IF(L220&gt;=K232,"Se Cumple","No se Cumple")</f>
-        <v>No se Cumple</v>
+        <v>Se Cumple</v>
       </c>
       <c r="T238">
         <v>70</v>
@@ -10193,11 +10193,11 @@
       </c>
       <c r="K239" s="86">
         <f>MAX(K236/K237,1)</f>
-        <v>1.09599802508861</v>
+        <v>1.09670537103314</v>
       </c>
       <c r="L239" s="86">
         <f>MAX(L236/L237,1)</f>
-        <v>1.02365634582899</v>
+        <v>1.00115447403687</v>
       </c>
       <c r="T239">
         <v>71</v>
@@ -10256,11 +10256,11 @@
       </c>
       <c r="K241" s="86">
         <f>IF(K226/K220&lt;1,"N/A",K226/K220)</f>
-        <v>1.09599802508861</v>
+        <v>1.09670537103314</v>
       </c>
       <c r="L241" s="86">
         <f>IF(L226/L220&lt;1,"N/A",L226/L220)</f>
-        <v>1.02365634582899</v>
+        <v>1.00115447403687</v>
       </c>
       <c r="T241">
         <v>73</v>
@@ -10316,11 +10316,11 @@
     <row r="243" spans="2:27" x14ac:dyDescent="0.3">
       <c r="K243" s="53">
         <f>K225/K220</f>
-        <v>1.21777558343179</v>
+        <v>1.21856152337015</v>
       </c>
       <c r="L243" s="53">
         <f>L225/L220</f>
-        <v>1.13739593980998</v>
+        <v>1.11239386004097</v>
       </c>
       <c r="T243">
         <v>75</v>

</xml_diff>